<commit_message>
version alineada al tema de tesis
</commit_message>
<xml_diff>
--- a/output/analisis_dimensional/00_resumen_ejecucion_pipeline.xlsx
+++ b/output/analisis_dimensional/00_resumen_ejecucion_pipeline.xlsx
@@ -427,7 +427,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -485,16 +485,16 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:07</t>
+          <t>2026-08-08T12:21:35</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:13</t>
+          <t>2026-08-08T12:21:41</t>
         </is>
       </c>
       <c r="F2" t="n">
-        <v>6.855</v>
+        <v>6.038</v>
       </c>
       <c r="G2" t="inlineStr">
         <is>
@@ -520,16 +520,16 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:13</t>
+          <t>2026-08-08T12:21:41</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:23</t>
+          <t>2026-08-08T12:21:50</t>
         </is>
       </c>
       <c r="F3" t="n">
-        <v>9.927</v>
+        <v>9.097</v>
       </c>
       <c r="G3" t="inlineStr">
         <is>
@@ -555,16 +555,16 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:23</t>
+          <t>2026-08-08T12:21:50</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:28</t>
+          <t>2026-08-08T12:21:54</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>4.638</v>
+        <v>4.025</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -590,16 +590,16 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:28</t>
+          <t>2026-08-08T12:21:54</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:46</t>
+          <t>2026-08-08T12:22:04</t>
         </is>
       </c>
       <c r="F5" t="n">
-        <v>17.79</v>
+        <v>9.426</v>
       </c>
       <c r="G5" t="inlineStr">
         <is>
@@ -625,16 +625,16 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:46</t>
+          <t>2026-08-08T12:22:04</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:02</t>
+          <t>2026-08-08T12:23:53</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>75.95999999999999</v>
+        <v>109.706</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
@@ -660,16 +660,16 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:02</t>
+          <t>2026-08-08T12:23:53</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:12</t>
+          <t>2026-08-08T12:24:02</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>10.398</v>
+        <v>8.878</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -695,16 +695,16 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:12</t>
+          <t>2026-08-08T12:24:02</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-08T08:26:58</t>
+          <t>2026-08-08T12:27:27</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>226.188</v>
+        <v>204.995</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -730,16 +730,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>2026-08-08T08:26:58</t>
+          <t>2026-08-08T12:27:27</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-08T08:30:56</t>
+          <t>2026-08-08T12:30:01</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>237.606</v>
+        <v>153.255</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -765,16 +765,16 @@
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>2026-08-08T08:30:56</t>
+          <t>2026-08-08T12:30:01</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-08-08T08:36:56</t>
+          <t>2026-08-08T12:34:45</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>360.226</v>
+        <v>284.801</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -800,16 +800,16 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>2026-08-08T08:36:56</t>
+          <t>2026-08-08T12:34:45</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>2026-08-08T08:38:51</t>
+          <t>2026-08-08T12:38:21</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>114.506</v>
+        <v>215.288</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -835,18 +835,123 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>2026-08-08T08:38:51</t>
+          <t>2026-08-08T12:38:21</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>2026-08-08T08:40:23</t>
+          <t>2026-08-08T12:41:14</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>92.473</v>
+        <v>173.426</v>
       </c>
       <c r="G12" t="inlineStr">
+        <is>
+          <t>Etapa finalizada sin errores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>graficas_metodologia</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>correcto</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:41:14</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:22</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>127.715</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Etapa finalizada sin errores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>graficas_modelos</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>correcto</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:22</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:33</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>10.722</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Etapa finalizada sin errores.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>graficas_rnn</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>general</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>correcto</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:33</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:52</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>19.371</v>
+      </c>
+      <c r="G15" t="inlineStr">
         <is>
           <t>Etapa finalizada sin errores.</t>
         </is>
@@ -863,7 +968,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C13"/>
+  <dimension ref="A1:C157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -886,180 +991,2340 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>00_manifiesto_pipeline.json</t>
+          <t>00_alineacion_investigacion.md</t>
         </is>
       </c>
       <c r="B2" t="n">
-        <v>5152</v>
+        <v>2665</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>2026-08-06T22:30:46</t>
+          <t>2026-08-08T12:43:52</t>
         </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>00_resumen_ejecucion_pipeline.xlsx</t>
+          <t>00_interpretacion_resultados_tesis.md</t>
         </is>
       </c>
       <c r="B3" t="n">
-        <v>7266</v>
+        <v>4627</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>2026-08-06T22:30:46</t>
+          <t>2026-08-08T12:25:38</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>01_perfil_dataset_y_dimensiones.xlsx</t>
+          <t>00_manifiesto_pipeline.json</t>
         </is>
       </c>
       <c r="B4" t="n">
-        <v>30709</v>
+        <v>27110</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:28</t>
+          <t>2026-08-08T12:15:08</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>02_diagnostico_multicolinealidad.xlsx</t>
+          <t>00_mejores_configuraciones_globales_modelos.json</t>
         </is>
       </c>
       <c r="B5" t="n">
-        <v>35497</v>
+        <v>1760</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>2026-08-08T08:21:46</t>
+          <t>2026-08-08T12:34:45</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>03_dataset_reducido_por_seleccion.xlsx</t>
+          <t>00_mejores_configuraciones_globales_modelos.xlsx</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>1908551</v>
+        <v>7238</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:02</t>
+          <t>2026-08-08T12:34:45</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>04_dataset_pca_componentes.xlsx</t>
+          <t>00_mejores_configuraciones_globales_rnn_lstm.json</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>3182843</v>
+        <v>2160</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>2026-08-08T08:23:12</t>
+          <t>2026-08-08T12:41:14</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>05_modelos_rolling_origin_completo.xlsx</t>
+          <t>00_mejores_configuraciones_globales_rnn_lstm.xlsx</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>44478</v>
+        <v>7590</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>2026-08-08T08:26:58</t>
+          <t>2026-08-08T12:41:14</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>05_modelos_rolling_origin_pca.xlsx</t>
+          <t>00_resumen_ejecucion_pipeline.xlsx</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>44731</v>
+        <v>11652</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>2026-08-08T08:36:56</t>
+          <t>2026-08-08T12:15:08</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>05_modelos_rolling_origin_reducido.xlsx</t>
+          <t>01_perfil_dataset_y_dimensiones.xlsx</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>44367</v>
+        <v>30709</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>2026-08-08T08:30:56</t>
+          <t>2026-08-08T12:21:54</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>06_rnn_lstm_pca.xlsx</t>
+          <t>02_diagnostico_multicolinealidad.xlsx</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>5483</v>
+        <v>35498</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>2026-08-08T08:40:23</t>
+          <t>2026-08-08T12:22:04</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>06_rnn_lstm_reducido.xlsx</t>
+          <t>03_dataset_reducido_por_seleccion.xlsx</t>
         </is>
       </c>
       <c r="B12" t="n">
-        <v>5487</v>
+        <v>906845</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>2026-08-08T08:38:51</t>
+          <t>2026-08-08T12:23:53</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>04_dataset_pca_componentes.xlsx</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>3182844</v>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:24:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>05_modelos_rolling_origin_completo.xlsx</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>49523</v>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:27:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>05_modelos_rolling_origin_pca.xlsx</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>49851</v>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:34:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>05_modelos_rolling_origin_reducido.xlsx</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>49560</v>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:30:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>06_rnn_lstm_pca.xlsx</t>
+        </is>
+      </c>
+      <c r="B17" t="n">
+        <v>35487</v>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:41:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>06_rnn_lstm_reducido.xlsx</t>
+        </is>
+      </c>
+      <c r="B18" t="n">
+        <v>36227</v>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:38:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Conclusiones_y_recomendaciones.txt</t>
+        </is>
+      </c>
+      <c r="B19" t="n">
+        <v>2830</v>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:27:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Discusion.txt</t>
+        </is>
+      </c>
+      <c r="B20" t="n">
+        <v>3586</v>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:26:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Documento_tesis_profesional.txt</t>
+        </is>
+      </c>
+      <c r="B21" t="n">
+        <v>11666</v>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:28:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Documento_tesis_word.txt</t>
+        </is>
+      </c>
+      <c r="B22" t="n">
+        <v>11465</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\01_cobertura_temporal_fuentes.png</t>
+        </is>
+      </c>
+      <c r="B23" t="n">
+        <v>78776</v>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\02_evolucion_inpc.png</t>
+        </is>
+      </c>
+      <c r="B24" t="n">
+        <v>130843</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\03_factor_ajuste_inflacion.png</t>
+        </is>
+      </c>
+      <c r="B25" t="n">
+        <v>139845</v>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\04_temperatura_promedio_hidalgo.png</t>
+        </is>
+      </c>
+      <c r="B26" t="n">
+        <v>164415</v>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\05_distribucion_categorias_clima.png</t>
+        </is>
+      </c>
+      <c r="B27" t="n">
+        <v>61317</v>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\06_eventos_festivos_fechas_pago.png</t>
+        </is>
+      </c>
+      <c r="B28" t="n">
+        <v>162037</v>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:08</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\07_serie_diaria_ventas_reales.png</t>
+        </is>
+      </c>
+      <c r="B29" t="n">
+        <v>254107</v>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\08_ventas_nominales_vs_reales.png</t>
+        </is>
+      </c>
+      <c r="B30" t="n">
+        <v>235194</v>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\09_distribucion_ventas_diarias.png</t>
+        </is>
+      </c>
+      <c r="B31" t="n">
+        <v>68064</v>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\10_ventas_por_dia_semana.png</t>
+        </is>
+      </c>
+      <c r="B32" t="n">
+        <v>63138</v>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:11</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\11_mapa_calor_ventas_mes_anio.png</t>
+        </is>
+      </c>
+      <c r="B33" t="n">
+        <v>83893</v>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\12_composicion_productos_vendidos.png</t>
+        </is>
+      </c>
+      <c r="B34" t="n">
+        <v>58341</v>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:12</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\13_margen_ganancia_mensual.png</t>
+        </is>
+      </c>
+      <c r="B35" t="n">
+        <v>154109</v>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\14_serie_diaria_compras_reales.png</t>
+        </is>
+      </c>
+      <c r="B36" t="n">
+        <v>225927</v>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:14</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\15_compras_por_clasificacion.png</t>
+        </is>
+      </c>
+      <c r="B37" t="n">
+        <v>86727</v>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:15</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\16_pareto_proveedores.png</t>
+        </is>
+      </c>
+      <c r="B38" t="n">
+        <v>157382</v>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\17_unidades_medida_normalizadas.png</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>60078</v>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:16</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\18_ventas_compras_mensuales.png</t>
+        </is>
+      </c>
+      <c r="B40" t="n">
+        <v>212440</v>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:17</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\19_saldo_operativo_mensual.png</t>
+        </is>
+      </c>
+      <c r="B41" t="n">
+        <v>70520</v>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:19</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\20_dias_sin_actividad.png</t>
+        </is>
+      </c>
+      <c r="B42" t="n">
+        <v>70241</v>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:20</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\21_valores_faltantes_dataset_maestro.png</t>
+        </is>
+      </c>
+      <c r="B43" t="n">
+        <v>123902</v>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:21</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\22_correlacion_variables_clave_maestro.png</t>
+        </is>
+      </c>
+      <c r="B44" t="n">
+        <v>288860</v>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\23_familias_ingenieria_caracteristicas.png</t>
+        </is>
+      </c>
+      <c r="B45" t="n">
+        <v>102902</v>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\24_expansion_dimensional_feature_engineering.png</t>
+        </is>
+      </c>
+      <c r="B46" t="n">
+        <v>56330</v>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:27</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\25_historial_minimo_y_observaciones.png</t>
+        </is>
+      </c>
+      <c r="B47" t="n">
+        <v>92566</v>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:32</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\26_codificacion_ciclica_mes.png</t>
+        </is>
+      </c>
+      <c r="B48" t="n">
+        <v>102216</v>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\27_codificacion_ciclica_dia_semana.png</t>
+        </is>
+      </c>
+      <c r="B49" t="n">
+        <v>118628</v>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\28_alineacion_rezago_7_dias.png</t>
+        </is>
+      </c>
+      <c r="B50" t="n">
+        <v>230419</v>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\29_correlacion_objetivo_rezagos.png</t>
+        </is>
+      </c>
+      <c r="B51" t="n">
+        <v>63783</v>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\30_comparacion_ventanas_moviles.png</t>
+        </is>
+      </c>
+      <c r="B52" t="n">
+        <v>225028</v>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\31_estadisticos_moviles_28_dias.png</t>
+        </is>
+      </c>
+      <c r="B53" t="n">
+        <v>244848</v>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:25:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\32_proximidad_fechas_pago.png</t>
+        </is>
+      </c>
+      <c r="B54" t="n">
+        <v>325265</v>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:04</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\33_ventanas_eventos_7_30_dias.png</t>
+        </is>
+      </c>
+      <c r="B55" t="n">
+        <v>205393</v>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\34_recencia_ventas_compras.png</t>
+        </is>
+      </c>
+      <c r="B56" t="n">
+        <v>151217</v>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\35_indicadores_financieros_derivados_7d.png</t>
+        </is>
+      </c>
+      <c r="B57" t="n">
+        <v>166176</v>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:18</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\36_relacion_media7_objetivo_ventas.png</t>
+        </is>
+      </c>
+      <c r="B58" t="n">
+        <v>159107</v>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:23</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\37_correlacion_features_objetivos.png</t>
+        </is>
+      </c>
+      <c r="B59" t="n">
+        <v>314042</v>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:28</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\38_esparsidad_features_modelado.png</t>
+        </is>
+      </c>
+      <c r="B60" t="n">
+        <v>166192</v>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\39_estructura_general_dataset_modelado.png</t>
+        </is>
+      </c>
+      <c r="B61" t="n">
+        <v>96345</v>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:33</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\40_variables_por_dimension_metodologica.png</t>
+        </is>
+      </c>
+      <c r="B62" t="n">
+        <v>104329</v>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\41_esparsidad_promedio_por_dimension.png</t>
+        </is>
+      </c>
+      <c r="B63" t="n">
+        <v>110409</v>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\42_nulos_promedio_por_dimension.png</t>
+        </is>
+      </c>
+      <c r="B64" t="n">
+        <v>94703</v>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:34</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\43_variables_constantes_por_dimension.png</t>
+        </is>
+      </c>
+      <c r="B65" t="n">
+        <v>101434</v>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\44_cardinalidad_vs_esparsidad_variables.png</t>
+        </is>
+      </c>
+      <c r="B66" t="n">
+        <v>181637</v>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\45_variables_mayor_concentracion_ceros.png</t>
+        </is>
+      </c>
+      <c r="B67" t="n">
+        <v>161795</v>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:36</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\46_coeficiente_variacion_variables.png</t>
+        </is>
+      </c>
+      <c r="B68" t="n">
+        <v>146866</v>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\47_rango_intercuartil_variables.png</t>
+        </is>
+      </c>
+      <c r="B69" t="n">
+        <v>156463</v>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:37</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\48_boxplot_resumen_objetivos.png</t>
+        </is>
+      </c>
+      <c r="B70" t="n">
+        <v>79100</v>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\49_intermitencia_variables_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B71" t="n">
+        <v>71085</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\50_matriz_calidad_dimensiones.png</t>
+        </is>
+      </c>
+      <c r="B72" t="n">
+        <v>143847</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\51_distribucion_correlaciones_altas.png</t>
+        </is>
+      </c>
+      <c r="B73" t="n">
+        <v>72560</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\52_pares_predictores_mayor_correlacion.png</t>
+        </is>
+      </c>
+      <c r="B74" t="n">
+        <v>251342</v>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\53_red_redundancia_predictores.png</t>
+        </is>
+      </c>
+      <c r="B75" t="n">
+        <v>167645</v>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\54_frecuencia_variables_redundantes.png</t>
+        </is>
+      </c>
+      <c r="B76" t="n">
+        <v>114759</v>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\55_conservadas_eliminadas_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B77" t="n">
+        <v>65225</v>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\56_dimensiones_conservadas_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B78" t="n">
+        <v>141467</v>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\57_relevancia_conservada_vs_eliminada.png</t>
+        </is>
+      </c>
+      <c r="B79" t="n">
+        <v>208628</v>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\58_ganancia_relevancia_filtro.png</t>
+        </is>
+      </c>
+      <c r="B80" t="n">
+        <v>66978</v>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\59_ranking_vif_variables.png</t>
+        </is>
+      </c>
+      <c r="B81" t="n">
+        <v>171276</v>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\60_clasificacion_variables_vif.png</t>
+        </is>
+      </c>
+      <c r="B82" t="n">
+        <v>59699</v>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\61_solapamiento_variables_eliminadas.png</t>
+        </is>
+      </c>
+      <c r="B83" t="n">
+        <v>52864</v>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\62_resumen_diagnostico_multicolinealidad.png</t>
+        </is>
+      </c>
+      <c r="B84" t="n">
+        <v>86126</v>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\63_resultado_global_seleccion_caracteristicas.png</t>
+        </is>
+      </c>
+      <c r="B85" t="n">
+        <v>92606</v>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\64_variables_seleccionadas_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B86" t="n">
+        <v>70655</v>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\65_distribucion_score_compuesto_seleccion.png</t>
+        </is>
+      </c>
+      <c r="B87" t="n">
+        <v>58964</v>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\66_top_caracteristicas_score_compuesto.png</t>
+        </is>
+      </c>
+      <c r="B88" t="n">
+        <v>526901</v>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:48</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\67_matriz_scores_metodos_top_variables.png</t>
+        </is>
+      </c>
+      <c r="B89" t="n">
+        <v>251785</v>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:49</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\68_concordancia_metodos_seleccion.png</t>
+        </is>
+      </c>
+      <c r="B90" t="n">
+        <v>138657</v>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:50</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\69_dimensiones_seleccionadas_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B91" t="n">
+        <v>142672</v>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:51</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\70_solapamiento_seleccion_entre_objetivos.png</t>
+        </is>
+      </c>
+      <c r="B92" t="n">
+        <v>58357</v>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\71_curvas_score_por_ranking.png</t>
+        </is>
+      </c>
+      <c r="B93" t="n">
+        <v>187599</v>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\72_esparsidad_coeficientes_lasso.png</t>
+        </is>
+      </c>
+      <c r="B94" t="n">
+        <v>72727</v>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:53</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\73_metodo_dominante_por_variable_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B95" t="n">
+        <v>67531</v>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:54</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\74_comparacion_dataset_completo_reducido.png</t>
+        </is>
+      </c>
+      <c r="B96" t="n">
+        <v>99015</v>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:55</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\75_reduccion_dimensional_pca.png</t>
+        </is>
+      </c>
+      <c r="B97" t="n">
+        <v>81531</v>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\76_scree_plot_pca.png</t>
+        </is>
+      </c>
+      <c r="B98" t="n">
+        <v>92703</v>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\77_varianza_acumulada_pca.png</t>
+        </is>
+      </c>
+      <c r="B99" t="n">
+        <v>110251</v>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\78_contribucion_primeros_componentes.png</t>
+        </is>
+      </c>
+      <c r="B100" t="n">
+        <v>55326</v>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\79_componentes_por_umbral_varianza.png</t>
+        </is>
+      </c>
+      <c r="B101" t="n">
+        <v>68020</v>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:26:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\80_mapa_cargas_primeros_componentes.png</t>
+        </is>
+      </c>
+      <c r="B102" t="n">
+        <v>106902</v>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\81_cargas_primer_componente.png</t>
+        </is>
+      </c>
+      <c r="B103" t="n">
+        <v>146152</v>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\82_contribucion_variables_primeros_componentes.png</t>
+        </is>
+      </c>
+      <c r="B104" t="n">
+        <v>96833</v>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\83_series_temporales_componentes_pca.png</t>
+        </is>
+      </c>
+      <c r="B105" t="n">
+        <v>458513</v>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:05</t>
+        </is>
+      </c>
+    </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\84_plano_factorial_pca1_pca2.png</t>
+        </is>
+      </c>
+      <c r="B106" t="n">
+        <v>534503</v>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:07</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\85_correlacion_componentes_objetivos.png</t>
+        </is>
+      </c>
+      <c r="B107" t="n">
+        <v>227549</v>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:10</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\86_ortogonalidad_componentes_pca.png</t>
+        </is>
+      </c>
+      <c r="B108" t="n">
+        <v>106540</v>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\generacion_metodologia_pca.log</t>
+        </is>
+      </c>
+      <c r="B109" t="n">
+        <v>8600</v>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\INDICE_GRAFICAS_METODOLOGIA_PCA.csv</t>
+        </is>
+      </c>
+      <c r="B110" t="n">
+        <v>57425</v>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\MANIFIESTO_METODOLOGIA_PCA.json</t>
+        </is>
+      </c>
+      <c r="B111" t="n">
+        <v>88662</v>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\MANIFIESTO_METODOLOGIA_PCA.md</t>
+        </is>
+      </c>
+      <c r="B112" t="n">
+        <v>81133</v>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:13</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>graficas_metodologia\RESUMEN_ESTADISTICO_METODOLOGIA_PCA.xlsx</t>
+        </is>
+      </c>
+      <c r="B113" t="n">
+        <v>4194828</v>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:35</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\01_particion_temporal_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B114" t="n">
+        <v>81554</v>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\02_ventana_supervisada_28_dias.png</t>
+        </is>
+      </c>
+      <c r="B115" t="n">
+        <v>69151</v>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\03_arquitectura_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B116" t="n">
+        <v>61209</v>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\04_dimensionalidad_entrada_recurrente.png</t>
+        </is>
+      </c>
+      <c r="B117" t="n">
+        <v>64807</v>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\05_comparacion_rmse_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B118" t="n">
+        <v>198626</v>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:57</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\06_comparacion_mae_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B119" t="n">
+        <v>200819</v>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:58</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\07_diagnostico_mape_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B120" t="n">
+        <v>215076</v>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\08_arquitectura_ganadora_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B121" t="n">
+        <v>106609</v>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:59</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\09_mejora_lstm_vs_rnn.png</t>
+        </is>
+      </c>
+      <c r="B122" t="n">
+        <v>115494</v>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\10_efecto_dataset_reducido_vs_pca.png</t>
+        </is>
+      </c>
+      <c r="B123" t="n">
+        <v>106464</v>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\11_relacion_mae_rmse_redes.png</t>
+        </is>
+      </c>
+      <c r="B124" t="n">
+        <v>122574</v>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:01</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\12_score_multicriterio_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B125" t="n">
+        <v>201857</v>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\13_configuracion_entrenamiento_redes.png</t>
+        </is>
+      </c>
+      <c r="B126" t="n">
+        <v>79315</v>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:02</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\14_complejidad_parametros_vs_muestra.png</t>
+        </is>
+      </c>
+      <c r="B127" t="n">
+        <v>73542</v>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:06</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\15_intermitencia_objetivos_periodo_prueba.png</t>
+        </is>
+      </c>
+      <c r="B128" t="n">
+        <v>81088</v>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\16_resumen_experimento_rnn_lstm.png</t>
+        </is>
+      </c>
+      <c r="B129" t="n">
+        <v>67247</v>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\generacion_rnn_lstm.log</t>
+        </is>
+      </c>
+      <c r="B130" t="n">
+        <v>1357</v>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\INDICE_GRAFICAS_RNN_LSTM.csv</t>
+        </is>
+      </c>
+      <c r="B131" t="n">
+        <v>10839</v>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\MANIFIESTO_RNN_LSTM.json</t>
+        </is>
+      </c>
+      <c r="B132" t="n">
+        <v>16451</v>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\MANIFIESTO_RNN_LSTM.md</t>
+        </is>
+      </c>
+      <c r="B133" t="n">
+        <v>14190</v>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>graficas_rnn_lstm\RESUMEN_ESTADISTICO_RNN_LSTM.xlsx</t>
+        </is>
+      </c>
+      <c r="B134" t="n">
+        <v>14782</v>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:28:09</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\01_esquema_validacion_rolling_origin.png</t>
+        </is>
+      </c>
+      <c r="B135" t="n">
+        <v>75186</v>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\02_cobertura_origenes_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B136" t="n">
+        <v>78359</v>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:38</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\03_ranking_rmse_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B137" t="n">
+        <v>364904</v>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:39</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\04_mejor_modelo_por_dataset_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B138" t="n">
+        <v>137340</v>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\05_mejora_frente_linea_base_empirica.png</t>
+        </is>
+      </c>
+      <c r="B139" t="n">
+        <v>190838</v>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:40</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\06_relacion_mae_rmse_modelos.png</t>
+        </is>
+      </c>
+      <c r="B140" t="n">
+        <v>300099</v>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:41</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\07_concordancia_rankings_metricas.png</t>
+        </is>
+      </c>
+      <c r="B141" t="n">
+        <v>81593</v>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:42</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\08_evolucion_temporal_rmse_ganadores.png</t>
+        </is>
+      </c>
+      <c r="B142" t="n">
+        <v>396414</v>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\09_distribucion_rmse_por_modelo.png</t>
+        </is>
+      </c>
+      <c r="B143" t="n">
+        <v>124633</v>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:43</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\10_estabilidad_modelos_cv_rmse.png</t>
+        </is>
+      </c>
+      <c r="B144" t="n">
+        <v>174434</v>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\11_ventanas_ganadas_por_modelo.png</t>
+        </is>
+      </c>
+      <c r="B145" t="n">
+        <v>66797</v>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:44</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\12_sensibilidad_modelos_dataset.png</t>
+        </is>
+      </c>
+      <c r="B146" t="n">
+        <v>109478</v>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\13_empirico_vs_modelos_avanzados.png</t>
+        </is>
+      </c>
+      <c r="B147" t="n">
+        <v>158282</v>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:45</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\14_diagnostico_mape_por_objetivo.png</t>
+        </is>
+      </c>
+      <c r="B148" t="n">
+        <v>202740</v>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\15_origenes_temporales_mas_dificiles.png</t>
+        </is>
+      </c>
+      <c r="B149" t="n">
+        <v>172721</v>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:46</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\16_score_multicriterio_modelos.png</t>
+        </is>
+      </c>
+      <c r="B150" t="n">
+        <v>170548</v>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\generacion_rolling_origin.log</t>
+        </is>
+      </c>
+      <c r="B151" t="n">
+        <v>1378</v>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\INDICE_GRAFICAS_ROLLING_ORIGIN.csv</t>
+        </is>
+      </c>
+      <c r="B152" t="n">
+        <v>12067</v>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="153">
+      <c r="A153" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\MANIFIESTO_ROLLING_ORIGIN.json</t>
+        </is>
+      </c>
+      <c r="B153" t="n">
+        <v>17619</v>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\MANIFIESTO_ROLLING_ORIGIN.md</t>
+        </is>
+      </c>
+      <c r="B154" t="n">
+        <v>15905</v>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>graficas_rolling_origin\RESUMEN_ESTADISTICO_ROLLING_ORIGIN.xlsx</t>
+        </is>
+      </c>
+      <c r="B155" t="n">
+        <v>44476</v>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>2026-08-08T11:27:47</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
           <t>pipeline_tesis.log</t>
         </is>
       </c>
-      <c r="B13" t="n">
-        <v>3354</v>
-      </c>
-      <c r="C13" t="inlineStr">
-        <is>
-          <t>2026-08-08T08:40:23</t>
+      <c r="B156" t="n">
+        <v>4096</v>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:43:52</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>Resultados.txt</t>
+        </is>
+      </c>
+      <c r="B157" t="n">
+        <v>2995</v>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>2026-08-08T12:26:13</t>
         </is>
       </c>
     </row>
@@ -1097,7 +3362,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>2026-08-08T08:40:23</t>
+          <t>2026-08-08T12:43:52</t>
         </is>
       </c>
     </row>

</xml_diff>